<commit_message>
Update README, holiday seed data, provisioning scripts and solution zips
- README follows the house template: calendar experience, theme and
  naming conventions, how holidays are calculated (observed-day rules
  per 5 U.S.C. 6103), deployment and known limitations
- Holidays.csv/.xlsx: fix "Veterans Day" and Washington's Birthday note
- Provisioning scripts now match the flow: FixedHoliday on Holidays;
  ISOWeekofYear, Quarter and FiscalYear on DateGenerator; list named
  "Holidays"; CSV path relative to the script
- Re-export DateGenerator 1.0.0.1 managed and unmanaged zips

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/Holidays.xlsx
+++ b/data/Holidays.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Brendan\Desktop\Projects\Date Generator\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\Projects\DateGenerator\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -91,9 +91,6 @@
     <t>Columbus Day</t>
   </si>
   <si>
-    <t>Veterns Day</t>
-  </si>
-  <si>
     <t>Always on the 11th</t>
   </si>
   <si>
@@ -115,9 +112,6 @@
     <t>Third Monday in January</t>
   </si>
   <si>
-    <t>Third Thursday in February</t>
-  </si>
-  <si>
     <t>The last Monday in May. Note: The week number may vary as May can have 4 or 5 weeks.</t>
   </si>
   <si>
@@ -155,6 +149,12 @@
   </si>
   <si>
     <t>FixedHoliday</t>
+  </si>
+  <si>
+    <t>Third Monday in February</t>
+  </si>
+  <si>
+    <t>Veterans Day</t>
   </si>
 </sst>
 </file>
@@ -1765,10 +1765,10 @@
         <v>16</v>
       </c>
       <c r="F1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G1" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="H1" t="s">
         <v>17</v>
@@ -1791,18 +1791,18 @@
         <v>0</v>
       </c>
       <c r="F2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G2" t="b">
         <v>1</v>
       </c>
       <c r="H2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B3" s="3">
         <v>1</v>
@@ -1817,18 +1817,18 @@
         <v>2</v>
       </c>
       <c r="F3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G3" t="b">
         <v>0</v>
       </c>
       <c r="H3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B4" s="3">
         <v>2</v>
@@ -1843,13 +1843,13 @@
         <v>2</v>
       </c>
       <c r="F4" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G4" t="b">
         <v>0</v>
       </c>
       <c r="H4" t="s">
-        <v>31</v>
+        <v>43</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -1869,18 +1869,18 @@
         <v>2</v>
       </c>
       <c r="F5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G5" t="b">
         <v>0</v>
       </c>
       <c r="H5" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B6" s="3">
         <v>6</v>
@@ -1895,13 +1895,13 @@
         <v>2</v>
       </c>
       <c r="F6" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G6" t="b">
         <v>1</v>
       </c>
       <c r="H6" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
@@ -1921,13 +1921,13 @@
         <v>2</v>
       </c>
       <c r="F7" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G7" t="b">
         <v>1</v>
       </c>
       <c r="H7" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -1947,13 +1947,13 @@
         <v>2</v>
       </c>
       <c r="F8" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G8" t="b">
         <v>0</v>
       </c>
       <c r="H8" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
@@ -1973,18 +1973,18 @@
         <v>2</v>
       </c>
       <c r="F9" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G9" t="b">
         <v>0</v>
       </c>
       <c r="H9" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>23</v>
+        <v>44</v>
       </c>
       <c r="B10" s="3">
         <v>11</v>
@@ -1999,18 +1999,18 @@
         <v>0</v>
       </c>
       <c r="F10" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G10" t="b">
         <v>1</v>
       </c>
       <c r="H10" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B11" s="3">
         <v>11</v>
@@ -2025,18 +2025,18 @@
         <v>5</v>
       </c>
       <c r="F11" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G11" t="b">
         <v>0</v>
       </c>
       <c r="H11" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B12" s="3">
         <v>12</v>
@@ -2051,18 +2051,18 @@
         <v>0</v>
       </c>
       <c r="F12" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G12" t="b">
         <v>1</v>
       </c>
       <c r="H12" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B13" s="3">
         <v>1</v>
@@ -2077,13 +2077,13 @@
         <v>2</v>
       </c>
       <c r="F13" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G13" t="b">
         <v>1</v>
       </c>
       <c r="H13" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
   </sheetData>

</xml_diff>